<commit_message>
Update Danh sách VNSH03 lô 1000 nhận từ X-Force.xlsx
</commit_message>
<xml_diff>
--- a/5. Other/Danh sách VNSH03 lô 1000 nhận từ X-Force.xlsx
+++ b/5. Other/Danh sách VNSH03 lô 1000 nhận từ X-Force.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VNET\5. Other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7B8E0EC-5C7A-413F-9B23-95FE6C8ACD76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B4EC81-2075-442E-9594-0BF604CF78E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{DE03BF13-5A63-4E6D-9BDA-D95C0EEDDB32}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="764" uniqueCount="275">
   <si>
     <t>STT</t>
   </si>
@@ -831,9 +831,6 @@
     <t>SL lỗi</t>
   </si>
   <si>
-    <t>Tồn SX</t>
-  </si>
-  <si>
     <t>Đã cho mượn</t>
   </si>
   <si>
@@ -844,6 +841,18 @@
   </si>
   <si>
     <t>16/10/26</t>
+  </si>
+  <si>
+    <t>Trả lại lỗi</t>
+  </si>
+  <si>
+    <t>Tồn thực tế</t>
+  </si>
+  <si>
+    <t>Tồn lỗi</t>
+  </si>
+  <si>
+    <t>180 chưa nhập ID</t>
   </si>
 </sst>
 </file>
@@ -1036,7 +1045,7 @@
     <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1484,7 +1493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F4CE4C5-33C3-485C-9EF7-1623C4B890AF}">
-  <dimension ref="A1:K1001"/>
+  <dimension ref="A1:N1001"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" style="8" customWidth="1"/>
@@ -1495,11 +1504,12 @@
     <col min="6" max="6" width="29.7109375" style="9" customWidth="1"/>
     <col min="7" max="7" width="12.42578125" customWidth="1"/>
     <col min="8" max="8" width="14.140625" customWidth="1"/>
-    <col min="9" max="9" width="11.85546875" customWidth="1"/>
-    <col min="10" max="10" width="11.7109375" customWidth="1"/>
+    <col min="9" max="11" width="11.85546875" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="13" max="13" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1526,13 +1536,19 @@
         <v>266</v>
       </c>
       <c r="J1" s="24" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="K1" s="24" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+        <v>273</v>
+      </c>
+      <c r="L1" s="24" t="s">
+        <v>268</v>
+      </c>
+      <c r="M1" s="24" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -1553,22 +1569,33 @@
       </c>
       <c r="H2" s="23">
         <f>COUNTIFS(D2:D1001,"Đã nhập kho")</f>
-        <v>181</v>
+        <v>210</v>
       </c>
       <c r="I2" s="25">
         <f>COUNTIFS(D2:D1001,"Lỗi")</f>
         <v>19</v>
       </c>
-      <c r="J2" s="30">
+      <c r="J2" s="25">
+        <f>COUNTIFS(E2:E1001,"*Trả lại X-Force*")</f>
+        <v>10</v>
+      </c>
+      <c r="K2" s="25">
+        <f>SUM(I2-J2)</f>
+        <v>9</v>
+      </c>
+      <c r="L2" s="30">
         <f>COUNTIFS(D2:D1001,"Đã cho mượn")</f>
         <v>1</v>
       </c>
-      <c r="K2" s="31">
-        <f>G2-H2</f>
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M2" s="31">
+        <f>SUM(G2-(H2+J2+L2))</f>
+        <v>33</v>
+      </c>
+      <c r="N2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -1584,9 +1611,9 @@
       <c r="E3" s="10"/>
       <c r="F3" s="15"/>
       <c r="G3" s="7"/>
-      <c r="J3" s="7"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3" s="7"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -1603,7 +1630,7 @@
       <c r="F4" s="15"/>
       <c r="G4" s="7"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -1620,7 +1647,7 @@
       <c r="F5" s="15"/>
       <c r="G5" s="7"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -1637,7 +1664,7 @@
       <c r="F6" s="15"/>
       <c r="G6" s="7"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1654,7 +1681,7 @@
       <c r="F7" s="15"/>
       <c r="G7" s="7"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1671,7 +1698,7 @@
       <c r="F8" s="15"/>
       <c r="G8" s="7"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -1688,7 +1715,7 @@
       <c r="F9" s="15"/>
       <c r="G9" s="7"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -1705,7 +1732,7 @@
       <c r="F10" s="15"/>
       <c r="G10" s="7"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1722,7 +1749,7 @@
       <c r="F11" s="15"/>
       <c r="G11" s="7"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1739,7 +1766,7 @@
       <c r="F12" s="15"/>
       <c r="G12" s="7"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1756,7 +1783,7 @@
       <c r="F13" s="15"/>
       <c r="G13" s="7"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1773,7 +1800,7 @@
       <c r="F14" s="15"/>
       <c r="G14" s="7"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1790,7 +1817,7 @@
       <c r="F15" s="15"/>
       <c r="G15" s="7"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -4774,7 +4801,7 @@
         <v>166</v>
       </c>
       <c r="D201" s="28" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E201" s="29" t="s">
         <v>209</v>
@@ -4791,7 +4818,9 @@
       <c r="C202" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D202" s="3"/>
+      <c r="D202" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E202" s="10"/>
       <c r="F202" s="10"/>
     </row>
@@ -4805,7 +4834,9 @@
       <c r="C203" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D203" s="3"/>
+      <c r="D203" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E203" s="10"/>
       <c r="F203" s="10"/>
     </row>
@@ -4819,7 +4850,9 @@
       <c r="C204" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D204" s="3"/>
+      <c r="D204" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E204" s="10"/>
       <c r="F204" s="10"/>
     </row>
@@ -4833,7 +4866,9 @@
       <c r="C205" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D205" s="3"/>
+      <c r="D205" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E205" s="10"/>
       <c r="F205" s="10"/>
     </row>
@@ -4861,7 +4896,9 @@
       <c r="C207" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D207" s="3"/>
+      <c r="D207" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E207" s="10"/>
       <c r="F207" s="10"/>
     </row>
@@ -4875,7 +4912,9 @@
       <c r="C208" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D208" s="3"/>
+      <c r="D208" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E208" s="10"/>
       <c r="F208" s="10"/>
     </row>
@@ -4889,7 +4928,9 @@
       <c r="C209" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D209" s="3"/>
+      <c r="D209" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E209" s="10"/>
       <c r="F209" s="10"/>
     </row>
@@ -4903,7 +4944,9 @@
       <c r="C210" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D210" s="3"/>
+      <c r="D210" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E210" s="10"/>
       <c r="F210" s="10"/>
     </row>
@@ -4933,7 +4976,9 @@
       <c r="C212" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D212" s="3"/>
+      <c r="D212" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E212" s="10"/>
       <c r="F212" s="10"/>
     </row>
@@ -4961,7 +5006,9 @@
       <c r="C214" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D214" s="3"/>
+      <c r="D214" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E214" s="10"/>
       <c r="F214" s="10"/>
     </row>
@@ -4975,7 +5022,9 @@
       <c r="C215" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D215" s="3"/>
+      <c r="D215" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E215" s="10"/>
       <c r="F215" s="10"/>
     </row>
@@ -5049,7 +5098,9 @@
       <c r="C220" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D220" s="3"/>
+      <c r="D220" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E220" s="10"/>
       <c r="F220" s="10"/>
     </row>
@@ -5063,7 +5114,9 @@
       <c r="C221" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D221" s="3"/>
+      <c r="D221" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E221" s="10"/>
       <c r="F221" s="10"/>
     </row>
@@ -5077,7 +5130,9 @@
       <c r="C222" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D222" s="3"/>
+      <c r="D222" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E222" s="10"/>
       <c r="F222" s="10"/>
     </row>
@@ -5091,7 +5146,9 @@
       <c r="C223" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D223" s="3"/>
+      <c r="D223" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E223" s="10"/>
       <c r="F223" s="10"/>
     </row>
@@ -5105,7 +5162,9 @@
       <c r="C224" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D224" s="3"/>
+      <c r="D224" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E224" s="10"/>
       <c r="F224" s="10"/>
     </row>
@@ -5135,7 +5194,9 @@
       <c r="C226" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D226" s="3"/>
+      <c r="D226" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E226" s="10"/>
       <c r="F226" s="10"/>
     </row>
@@ -5149,7 +5210,9 @@
       <c r="C227" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D227" s="3"/>
+      <c r="D227" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E227" s="10"/>
       <c r="F227" s="10"/>
     </row>
@@ -5225,7 +5288,9 @@
       <c r="C232" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D232" s="3"/>
+      <c r="D232" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E232" s="10"/>
       <c r="F232" s="10"/>
     </row>
@@ -5269,7 +5334,9 @@
       <c r="C235" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D235" s="3"/>
+      <c r="D235" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E235" s="10"/>
       <c r="F235" s="10"/>
     </row>
@@ -5297,7 +5364,9 @@
       <c r="C237" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D237" s="3"/>
+      <c r="D237" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E237" s="10"/>
       <c r="F237" s="10"/>
     </row>
@@ -5371,7 +5440,9 @@
       <c r="C242" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D242" s="3"/>
+      <c r="D242" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E242" s="10"/>
       <c r="F242" s="10"/>
     </row>
@@ -5385,7 +5456,9 @@
       <c r="C243" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D243" s="3"/>
+      <c r="D243" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E243" s="10"/>
       <c r="F243" s="10"/>
     </row>
@@ -5461,7 +5534,9 @@
       <c r="C248" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D248" s="3"/>
+      <c r="D248" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E248" s="10"/>
       <c r="F248" s="10"/>
     </row>
@@ -5475,7 +5550,9 @@
       <c r="C249" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D249" s="3"/>
+      <c r="D249" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E249" s="10"/>
       <c r="F249" s="10"/>
     </row>
@@ -5489,7 +5566,9 @@
       <c r="C250" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D250" s="3"/>
+      <c r="D250" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E250" s="10"/>
       <c r="F250" s="10"/>
     </row>
@@ -5517,7 +5596,9 @@
       <c r="C252" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D252" s="3"/>
+      <c r="D252" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E252" s="10"/>
       <c r="F252" s="10"/>
     </row>
@@ -5545,7 +5626,9 @@
       <c r="C254" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D254" s="3"/>
+      <c r="D254" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E254" s="10"/>
       <c r="F254" s="10"/>
     </row>
@@ -5559,7 +5642,9 @@
       <c r="C255" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D255" s="3"/>
+      <c r="D255" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E255" s="10"/>
       <c r="F255" s="10"/>
     </row>
@@ -5568,10 +5653,10 @@
         <v>255</v>
       </c>
       <c r="B256" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="C256" s="4" t="s">
         <v>270</v>
-      </c>
-      <c r="C256" s="4" t="s">
-        <v>271</v>
       </c>
       <c r="D256" s="3"/>
       <c r="E256" s="10"/>

</xml_diff>